<commit_message>
update penelitian dan pkm data
</commit_message>
<xml_diff>
--- a/te-upgris/src/data/dummy/Hasil_Konversi_JSON.xlsx
+++ b/te-upgris/src/data/dummy/Hasil_Konversi_JSON.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MYDATA\Project\webte\te-upgris\src\data\dummy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DE6657A-3E28-475F-A8F5-6A65E67CABC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC92D08F-DF86-436B-B2F6-880A07AE6576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="beranda" sheetId="1" r:id="rId1"/>
@@ -27,12 +27,12 @@
     <sheet name="slideshow" sheetId="12" r:id="rId12"/>
     <sheet name="spmi" sheetId="13" r:id="rId13"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="539">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="672">
   <si>
     <t>videoUrl</t>
   </si>
@@ -400,12 +400,6 @@
     <t>Sistem Tenaga Listrik &amp; Smart Grid</t>
   </si>
   <si>
-    <t>S3 — Universitas Gadjah Mada</t>
-  </si>
-  <si>
-    <t>Sistem Tenaga Listrik, Analisis Sistem Daya, Pembangkit Energi Terbarukan</t>
-  </si>
-  <si>
     <t>PII, Sertifikasi Dosen</t>
   </si>
   <si>
@@ -427,15 +421,6 @@
     <t>Elektronika &amp; Sistem Kontrol</t>
   </si>
   <si>
-    <t>S2 — Institut Teknologi Bandung</t>
-  </si>
-  <si>
-    <t>Elektronika Daya, Sistem Kontrol Otomatis, PLC &amp; SCADA</t>
-  </si>
-  <si>
-    <t>BNSP Teknik Elektronika</t>
-  </si>
-  <si>
     <t>https://sinta.kemdikbud.go.id/authors/profile/123457</t>
   </si>
   <si>
@@ -445,15 +430,6 @@
     <t>Telekomunikasi &amp; Jaringan</t>
   </si>
   <si>
-    <t>S2 — Universitas Diponegoro</t>
-  </si>
-  <si>
-    <t>Sistem Telekomunikasi, Jaringan Komputer, Antena &amp; Propagasi</t>
-  </si>
-  <si>
-    <t>Cisco CCNA</t>
-  </si>
-  <si>
     <t>https://sinta.kemdikbud.go.id/authors/profile/123458</t>
   </si>
   <si>
@@ -463,15 +439,6 @@
     <t>Instrumentasi &amp; Pengukuran</t>
   </si>
   <si>
-    <t>S2 — Universitas Gadjah Mada</t>
-  </si>
-  <si>
-    <t>Instrumentasi Industri, Sensor &amp; Aktuator, Pengukuran Listrik</t>
-  </si>
-  <si>
-    <t>PII</t>
-  </si>
-  <si>
     <t>https://sinta.kemdikbud.go.id/authors/profile/123459</t>
   </si>
   <si>
@@ -484,12 +451,6 @@
     <t>Internet of Things &amp; Embedded Systems</t>
   </si>
   <si>
-    <t>S2 — Universitas Indonesia</t>
-  </si>
-  <si>
-    <t>Mikrokontroler &amp; Embedded System, IoT, Pemrograman Sistem Tertanam</t>
-  </si>
-  <si>
     <t>BNSP IoT</t>
   </si>
   <si>
@@ -502,15 +463,6 @@
     <t>Energi Terbarukan &amp; Efisiensi Energi</t>
   </si>
   <si>
-    <t>S2 — Institut Teknologi Sepuluh Nopember</t>
-  </si>
-  <si>
-    <t>Energi Terbarukan, Konservasi Energi, Panel Surya &amp; PLTS</t>
-  </si>
-  <si>
-    <t>Auditor Energi BNSP</t>
-  </si>
-  <si>
     <t>https://sinta.kemdikbud.go.id/authors/profile/123461</t>
   </si>
   <si>
@@ -520,12 +472,6 @@
     <t>Robotika &amp; Otomasi</t>
   </si>
   <si>
-    <t>Robotika, Otomasi Industri, Mekatronika</t>
-  </si>
-  <si>
-    <t>BNSP Robotik</t>
-  </si>
-  <si>
     <t>https://sinta.kemdikbud.go.id/authors/profile/123462</t>
   </si>
   <si>
@@ -535,12 +481,6 @@
     <t>Kecerdasan Buatan &amp; Pemrosesan Sinyal</t>
   </si>
   <si>
-    <t>Pemrosesan Sinyal Digital, Kecerdasan Buatan, Machine Learning untuk Teknik</t>
-  </si>
-  <si>
-    <t>Google TensorFlow Developer</t>
-  </si>
-  <si>
     <t>https://sinta.kemdikbud.go.id/authors/profile/123463</t>
   </si>
   <si>
@@ -997,67 +937,16 @@
     <t>roadmap</t>
   </si>
   <si>
-    <t>Optimasi Smart Grid Berbasis Algoritma Particle Swarm Optimization untuk Distribusi Energi Terbarukan</t>
-  </si>
-  <si>
-    <t>Dr Adhi Kusmanto, S.T., M.Eng.</t>
-  </si>
-  <si>
     <t>TS</t>
   </si>
   <si>
-    <t>Rp 85.000.000</t>
-  </si>
-  <si>
     <t>Dikti</t>
   </si>
   <si>
-    <t>Sistem Energi Cerdas</t>
-  </si>
-  <si>
-    <t>https://images.unsplash.com/photo-1473341304170-971dccb5ac1e?w=600&amp;q=70</t>
-  </si>
-  <si>
-    <t>/content/penelitian/penelitian-1.md</t>
-  </si>
-  <si>
-    <t>Sistem Monitoring Kualitas Daya Listrik Berbasis IoT untuk Industri Manufaktur</t>
-  </si>
-  <si>
-    <t>Rp 60.000.000</t>
-  </si>
-  <si>
     <t>Internal Lembaga</t>
   </si>
   <si>
-    <t>Otomasi Industri</t>
-  </si>
-  <si>
-    <t>https://images.unsplash.com/photo-1581092921461-7031e4bfb83e?w=600&amp;q=70</t>
-  </si>
-  <si>
-    <t>Pengembangan Robot Inspeksi Saluran Tegangan Tinggi dengan Computer Vision</t>
-  </si>
-  <si>
     <t>TS-1</t>
-  </si>
-  <si>
-    <t>Rp 75.000.000</t>
-  </si>
-  <si>
-    <t>https://images.unsplash.com/photo-1485827404703-89b55fcc595e?w=600&amp;q=70</t>
-  </si>
-  <si>
-    <t>/content/penelitian/penelitian-3.md</t>
-  </si>
-  <si>
-    <t>Klasifikasi Gangguan Sistem Tenaga Listrik Menggunakan Deep Learning</t>
-  </si>
-  <si>
-    <t>Rp 50.000.000</t>
-  </si>
-  <si>
-    <t>AI untuk Sistem Tenaga</t>
   </si>
   <si>
     <t>deskripsi</t>
@@ -1653,6 +1542,532 @@
   </si>
   <si>
     <t>0608108204</t>
+  </si>
+  <si>
+    <t>Teknik Elektro, UGM / Tenaga Listrik</t>
+  </si>
+  <si>
+    <t>Teknik Elektro UGM / Sistem Kendali</t>
+  </si>
+  <si>
+    <t>Teknik Elektro, UGM / Jaringan Komputer</t>
+  </si>
+  <si>
+    <t>Teknik Elektro, UNDIP / Telekomunikasi</t>
+  </si>
+  <si>
+    <t>Fisika, UGM / Konversi Energi</t>
+  </si>
+  <si>
+    <t>Fisika, UGM / Material Teknik</t>
+  </si>
+  <si>
+    <t>Konversi Energi</t>
+  </si>
+  <si>
+    <t>Pembangkit Listrik Energi Terbarukan, Teknik Kontrol Digital, Metodologi Penelitian</t>
+  </si>
+  <si>
+    <t>Rangkaian Listrik,
+analisis Tenaga Listrik</t>
+  </si>
+  <si>
+    <t>Jaringan Komputer, Elektronika Digital, Matematika Diskret</t>
+  </si>
+  <si>
+    <t>Dasar Telekomunikasi, Pengolahan Citra, Teknologi Informasi, Antarmuka dan Arsitektur Komputer, Jaringan komputer</t>
+  </si>
+  <si>
+    <t>Pengolahan Citra, sensor tranduser</t>
+  </si>
+  <si>
+    <t>Bahan-bahan Listrik, Sensor dan Tranduser, Fisika Listrik</t>
+  </si>
+  <si>
+    <t>BNSP Tenaga Listrik</t>
+  </si>
+  <si>
+    <t>BNSP Otomasi Industri</t>
+  </si>
+  <si>
+    <t>PENGEMBANGAN STADIOMETER DIGITAL UNTUK DETEKSI DINI RISIKO STUNTING PADA ANAK-ANAK USIA DI BAWAH 5 TAHUN</t>
+  </si>
+  <si>
+    <t>DESAIN SISTEM KENDALI SUHU RUANG PEMANAS DENGAN METODE ULTIMATE CYCLE</t>
+  </si>
+  <si>
+    <t>EKSTRAKSI KARAGENAN RUMPUT LAUT (GRACILARIA GIGAS) MENGGUNAKAN METODE REFLUKS DAN PENGAPLIKASIANNYA PADA ENKAPSULAN EKSTRAK KULIT BUAH MANGGIS (GARCINIA MANGOSTANA L.)</t>
+  </si>
+  <si>
+    <t>PEMANFAATAN AERATOR BERPENGGERAK TURBIN SAVONIUS DARRIEUS UNTUK PENINGKATAN HASIL PRODUKSI PADA TAMBAK PEMBESARAN IKAN BANDENG (CHANOS CHANOS FORSKAL)</t>
+  </si>
+  <si>
+    <t>PENINGKATAN DAYA PV TERHUBUNG KE GRID DENGAN KOORDINASI KONTROL MPPT</t>
+  </si>
+  <si>
+    <t>DESAIN MODEL FUZZY LOGIC UNTUK PENILAIAN KUALITAS AIR SUMUR BERDASARKAN PARAMETER SALINITAS, PH, DAN KEKERUHAN DI SEMARANG</t>
+  </si>
+  <si>
+    <t>PENGELOLAAN BANJIR DENGAN SISTEM POLDER BERBASIS TEKNOLOGI INFORMASI DAN IOT</t>
+  </si>
+  <si>
+    <t>DESAIN MULTI-KONVERTER UNTUK PENGATURAN TEGANGAN DC MIKROGRID DENGAN FUZZY LOGIC</t>
+  </si>
+  <si>
+    <t>DESAIN BATERAI INVERTER SATU FASA DENGAN KONTROL PI-FUZZY UNTUK PENINGKATAN STABILITAS DAYA AC MIKROGRID</t>
+  </si>
+  <si>
+    <t>PRODUK INOVASI TEKNOLOGI HYBRID POMPA AIR MENGGUNAKAN INTERNET OF THING (IOT), WIND TURBINE DAN SOLAR PANEL SEBAGAI SALAH SATU SOLUSI PENGAIRAN AIR SAWAH DI WILAYAH DEMAK</t>
+  </si>
+  <si>
+    <t>OPTIMASI PENDINGIN TERMOAKUSTIK DENGAN TENAGA MESIN TERMOAKUSTIK MEMANFAATKAN LIMBAH PANAS DAN MATAHARI</t>
+  </si>
+  <si>
+    <t>Formulasi Pembelajaran Fisika Kontekstual Berorientasi Swasembada Energi Untuk Meningkatkan Literasi Energi Siswa</t>
+  </si>
+  <si>
+    <t>PENGEMBANGAN MEDIA PEMBELAJARAN FISIKA BERBASIS KERANGKA KERJA DEEP LEARNING UNTUK MENINGKATKAN MINAT BELAJAR DAN KEMAMPUAN PEMECAHAN MASALAH SISWA</t>
+  </si>
+  <si>
+    <t>RANCANG BANGUN PROTOTYPE ALAT UKUR POSISI BENDA BERBASIS CITRA STEREOSKOPIK</t>
+  </si>
+  <si>
+    <t>STUDY ON LOW SYMMETRY EFFECT OF A2BF6 CRYSTALS DOPED MN4+</t>
+  </si>
+  <si>
+    <t>TRACER STUDY PENDIDIKAN FISIKA UNIVERSITAS PGRI SEMARANG PADA ALUMNI LULUSAN TAHUN 2018-2022</t>
+  </si>
+  <si>
+    <t>PENGEMBANGAN E-LKPD BERBASIS MASALAH POKOK BAHASAN PENGUKURAN BESARAN FISIS UNTUK MENINGKATKAN PEMAHANAN KONSEP DAN KEMAMPUAN PENGAMBILAN KEPUTUSAN</t>
+  </si>
+  <si>
+    <t>PENGEMBANGAN E-LKPD BERBASIS PENYELESAIAN MASALAH PADA POKOK BAHASAN ENERGI TERBARUKAN UNTUK MENINGKATKAN PEMAHAMAN KONSEP DAN PENGAMBILAN KEPUTUSAN</t>
+  </si>
+  <si>
+    <t>PROFIL MINAT SISWA SLTA DALAM MELANJUTKAN STUDI DI PERGURAN TINGGI</t>
+  </si>
+  <si>
+    <t>PENERAPAN PROJEK BASED LEARNING (PJBL) UNTUK MENINGKATKAN KREATIVITAS DAN KETERAMPILAN KERJASAMA PESERTA DIDIK DALAM PEMBELAJARAN FISIKA</t>
+  </si>
+  <si>
+    <t>PREPARASI DAN OPTIMASI KETEBALAN LAPISAN TUNGGAL BAHAN NON MAGNETIK ENCENG GONDOK MENGGUNAKAN MATLAB SEBAGAI RADAR ABSORBER MATERIAL</t>
+  </si>
+  <si>
+    <t>Studi Sifat Optik Fosfor Merah berbasis Hafnium (Hf) untuk White LED</t>
+  </si>
+  <si>
+    <t>PENGEMBANGAN ALAT PERAGA ENERGI TERBARUKAN BERBASIS IOT DENGAN PENDEKATAN ESD UNTUK MENINGKATKAN KETERAMPILAN GENERIK SAINS</t>
+  </si>
+  <si>
+    <t>Studi Pengaruh Jenis, Komposisi, dan Tekanan Gas Kerja Terhadap Kinerja Pembangkit Listrik Termoakustik</t>
+  </si>
+  <si>
+    <t>KONVERSI ENERGI PANAS MENJADI ENERGI AKUSTIK
+DARI MESIN TERMOAKUSTIK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pengembangan Peredam Panas Ramah Lingkungan pada Atap Bangunan Berbasis Serat Kelapa
+</t>
+  </si>
+  <si>
+    <t>Ekstraksi Karagenan Rumput Laut (Gracilaria gigas) Menggunakan Metode Refluks dan Pengaplikasiannya pada Enkapsulan Ekstrak Kulit Buah Manggis (Garcinia mangostana L.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PEMANFAATAN AERATOR BERPENGGERAK TURBIN SAVONIUS DARRIEUS UNTUK PENINGKATAN HASIL PRODUKSI PADA TAMBAK PEMBESARAN IKAN BANDENG (Chanos Chanos Forskal)
+</t>
+  </si>
+  <si>
+    <t>Rekayasa Formulasi Kerupuk Ikan Berbasis Kombinasi Daging Lele (Clarias sp.) dan Tenggiri (Scomberomorus sp.) serta Implikasinya terhadap Sifat Fisik, Kimia, dan Sensorik Produk</t>
+  </si>
+  <si>
+    <t>Preparasi, Karakterisasi, dan Optimasi Ketebalan Lapisan Tunggal Bahan Non Magnetik Sekam Padi sebagai Radar Absorber Material</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pengembangan Media Pembelajaran Fisika Berbasis Kerangka Kerja Deep Learning untuk Meningkatkan Minat Belajar dan Kemampuan Pemecahan Masalah Siswa
+</t>
+  </si>
+  <si>
+    <t>Pengaruh Pemberian Cat pada Atap Bangunan Terhadap Laju Transfer Panas</t>
+  </si>
+  <si>
+    <t>Rancang Bangun Prototype Alat Ukur Posisi Benda Berbasis Citra Stereoskopik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PREDICTING CRYSTAL SYSTEMS OF LI-ION BATTERY CATHODES USING MACHINE LEARNING
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pengembangan E-LKPD Berbasis Masalah Pokok Bahasan Pengukuran Besaran Fisis Untuk Meningkatkan Pemahanan Konsep dan Kemampuan Pengambilan Keputusan
+</t>
+  </si>
+  <si>
+    <t>Slamet Supriyadi REGULER ( PTH ) Margono; Bambang Hadi Kunaryo;</t>
+  </si>
+  <si>
+    <t>Ganjar Winasis REGULER ( DOSEN PEMULA ) Bambang Hadi Kunaryo;</t>
+  </si>
+  <si>
+    <t>Muhammad Amiruddin MANDIRI ( MANDIRI ) Imadudin Harjanto; Bambang Hadi Kunaryo; Affandi Faisal Kurniawan; Sigit Ristanto;</t>
+  </si>
+  <si>
+    <t>Rizky Muliani Dwi Ujianti REGULER - DASAR/FUNDAMENTAL ( REGULER - DASAR/FUNDAMENTAL ) Althesa Androva; Bambang Hadi Kunaryo;</t>
+  </si>
+  <si>
+    <t>Rizky Muliani Dwi Ujianti REGULER ( REG ) Althesa Androva; Bambang Hadi Kunaryo; Nur Aksin;</t>
+  </si>
+  <si>
+    <t>Adhi Kusmantoro PENELITIAN REGULER ( REGULER ) Bambang Hadi Kunaryo;</t>
+  </si>
+  <si>
+    <t>Agus Mukhtar REGULER ( DOSEN PEMULA ) Aan Burhanudin; Muhammad Amiruddin; Rifki Hermana;</t>
+  </si>
+  <si>
+    <t>Ikhwanudin PENELITIAN DESENTRALISASI ( PDUPT ) Farida Yudaningrum; Imadudin Harjanto;</t>
+  </si>
+  <si>
+    <t>Adhi Kusmantoro REGULER ( REG ) Irna Farikhah;</t>
+  </si>
+  <si>
+    <t>Adhi Kusmantoro  Irna Farikhah;</t>
+  </si>
+  <si>
+    <t>Achmad Buchori  Adhi Kusmantoro; Aan Burhanudin;</t>
+  </si>
+  <si>
+    <t>Irna Farikhah Harto Nuroso; Mega Novita;</t>
+  </si>
+  <si>
+    <t>Nur Khoiri Sigit Ristanto; Affandi Faisal Kurniawan;</t>
+  </si>
+  <si>
+    <t>Sigit Ristanto Nur Khoiri; Affandi Faisal Kurniawan;</t>
+  </si>
+  <si>
+    <t>Sigit RistantoNur Khoiri; Affandi Faisal Kurniawan;</t>
+  </si>
+  <si>
+    <t>Mega Novita Sigit Ristanto; Ernawati Saptaningrum; Slamet Supriyadi;</t>
+  </si>
+  <si>
+    <t>Sigit Ristanto Affandi Faisal Kurniawan; Ummi Kaltsum; Ernawati Saptaningrum;</t>
+  </si>
+  <si>
+    <t>Nur Khoiri Sapto Budoyo; Senowarsito; Sigit Ristanto;</t>
+  </si>
+  <si>
+    <t>Nur Khoiri Affandi Faisal Kurniawan; Joko Saefan;</t>
+  </si>
+  <si>
+    <t>Mega Novita Penelitian Kompetitif Nasional ( PFR )Rizky Muliani Dwi Ujianti; Affandi Faisal Kurniawan; Nur Latifah Dwi Mutiara Sari;</t>
+  </si>
+  <si>
+    <t>Affandi Faisal Kurniawan REGULER ( REGULER )Nur Khoiri; Joko Saefan;</t>
+  </si>
+  <si>
+    <t>IKHSAN SETIAWANAGUNG BAMBANG SETIO, PRASTOWO MURTI UTOMO, IRNA FARIKHAH</t>
+  </si>
+  <si>
+    <t>Irna FarikhahNur Khoiri, Setyoningsih Wibowo,</t>
+  </si>
+  <si>
+    <t>Dr SLAMET SUPRIYADI, M.Env.St.Margono, ST., M.Eng; Bambang Hadi Kunaryo, S.T., M.T.; Winda Margaretha; Silfia Dea Ananta; Sisilia Nava Brillian Angelica</t>
+  </si>
+  <si>
+    <t>Dr.Pi Rizky Muliani Dwi Ujianti, S.Pi., M.SiAlthesa Androva, S.T., M.Eng; Bambang Hadi Kunaryo, S.T., M.T.; CARISA ZAHRA AZURA; RIHMA NUR HAYATI; ALIFAH DWI SUSANTI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr.Pi Rizky Muliani Dwi Ujianti, S.Pi., M.Si
+Althesa Androva, S.T., M.Eng; Bambang Hadi Kunaryo, S.T., M.T.; Nur Aksin, S.Ag., M.SI; KHOIRUS SA`ADAH; LAILATUS SA'DIYAH SEPTIYANI; MUTIARA SABATINA PUTRIYANTO
+</t>
+  </si>
+  <si>
+    <t>Dr.Pi Rizky Muliani Dwi Ujianti, S.Pi., M.SiAlthesa Androva, S.T., M.Eng; Bambang Hadi Kunaryo, S.T., M.T.; MUTIARA FITRI RAHMANINGTYAS; ARINA AINI NURUL KHASANAH; Abdillah Fathan Generus Annajah</t>
+  </si>
+  <si>
+    <t>Dr. Affandi Faisal Kurniawan, S.Si.,M.Sc.Prof. Dr. Nur Khoiri, S.Pd., M.T., M.Pd.; Dr. Sigit Ristanto, ST., M.Sc; Joko Saefan, M. Sc.; Naifah Istya Putri Aprilia; Nadroti Hidayatun Ni’mah; Murtiningsih</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. Sigit Ristanto, ST., M.Sc
+Prof. Dr. Nur Khoiri, S.Pd., M.T., M.Pd.; Dr. Affandi Faisal Kurniawan, S.Si.,M.Sc.; Emila Luthfia Sofa; Julia; Dwi Amiliya Putri
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. Sigit Ristanto, ST., M.ScDr SLAMET SUPRIYADI, M.Env.St.; Dr. Baju Arie Wibawa, S.T., M.T; Winda Margaretha; Yunita Dwi Saputri Ome; Pramudhita Alfina Damayanti
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. Sigit Ristanto, ST., M.ScProf. Dr. Nur Khoiri, S.Pd., M.T., M.Pd.; Dr. Affandi Faisal Kurniawan, S.Si.,M.Sc.; Nur Roikhana Zulfa; Pramudhita Alfina Damayanti; Ratih Meiwulan
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr.Pi Rizky Muliani Dwi Ujianti, S.Pi., M.Si
+Dr. Sigit Ristanto, ST., M.Sc; Bambang Agus Herlambang, S.Kom., M.Kom; Rina Widyawati; Sri Wahyuni; Tri Ambarwati Mardikaningrum; Prof. Kazuyoshi Ogasawara
+</t>
+  </si>
+  <si>
+    <t> 2025  </t>
+  </si>
+  <si>
+    <t> 2024  </t>
+  </si>
+  <si>
+    <t> 2023  </t>
+  </si>
+  <si>
+    <t> 2021  </t>
+  </si>
+  <si>
+    <t> 2022  </t>
+  </si>
+  <si>
+    <t>Rp7,500,000.00</t>
+  </si>
+  <si>
+    <t>Rp10,000,000.00</t>
+  </si>
+  <si>
+    <t>Rp5,000,000.00</t>
+  </si>
+  <si>
+    <t>Rp9,000,000.00</t>
+  </si>
+  <si>
+    <t>Rp90,000,000.00</t>
+  </si>
+  <si>
+    <t>Rp6,500,000.00</t>
+  </si>
+  <si>
+    <t>Rp218,316,000.00</t>
+  </si>
+  <si>
+    <t>Rp20,000,000.00</t>
+  </si>
+  <si>
+    <t>Rp99,664,000.00</t>
+  </si>
+  <si>
+    <t>Rp132,060,000.00</t>
+  </si>
+  <si>
+    <t>Rp24,500,000.00</t>
+  </si>
+  <si>
+    <t>Rp15,000,000.00</t>
+  </si>
+  <si>
+    <t>Rp12,000,000.00</t>
+  </si>
+  <si>
+    <t>Rp12,500,000.00</t>
+  </si>
+  <si>
+    <t>Rp23,000,000.00</t>
+  </si>
+  <si>
+    <t>Rp50,000,000.00</t>
+  </si>
+  <si>
+    <t>LPPM</t>
+  </si>
+  <si>
+    <t>Mandiri</t>
+  </si>
+  <si>
+    <t>DRTPM</t>
+  </si>
+  <si>
+    <t>PENELITIAN KOMPETITIF NASIONAL ( PENELITIAN TERAPAN KOMPETITIF NASIONAL )</t>
+  </si>
+  <si>
+    <t>HIBAH APBU ( APBU )</t>
+  </si>
+  <si>
+    <t> PENELITIAN DESENTRALISASI ( PDUPT )</t>
+  </si>
+  <si>
+    <t>Penelitian Kompetitif Nasional ( PFR )</t>
+  </si>
+  <si>
+    <t>REGULER ( PTH )</t>
+  </si>
+  <si>
+    <t> REGULER ( REG )</t>
+  </si>
+  <si>
+    <t>KERJASAMA LUAR NEGERI ( KLN )</t>
+  </si>
+  <si>
+    <t>PENUGASAN ( PENUGASAN )</t>
+  </si>
+  <si>
+    <t>HIBAH APBU ( HIBAH APBU )</t>
+  </si>
+  <si>
+    <t>REGULER ( PTK )</t>
+  </si>
+  <si>
+    <t>lPPM</t>
+  </si>
+  <si>
+    <t>PROGRAM PENELITIAN INTERNAL 
+SKEMA KERJASAMA LUAR NEGERI</t>
+  </si>
+  <si>
+    <t>Reguler</t>
+  </si>
+  <si>
+    <t>PKM PROGRAM PERBAIKAN DAN EDUKASI PENGGUNAAN PERALATAN AUDIO BAGI PANTI ASUHAN FACHRUDIN SEMARANG</t>
+  </si>
+  <si>
+    <t>PKM KELOMPOK PEMBUDIDAYA LELE: TEKNOLOGI ZERO WASTE AIR LIMBAH KOLAM BERBASIS IOT UNTUK PENINGKATAN PRODUKSI DAN PENCEGAHAN STUNTING PADA ANAK</t>
+  </si>
+  <si>
+    <t>PKM PENDAMPINGAN INSTALASI SISTEM CCTV UNTUK MASJID BAITUL ROHMAH PUDAK PAYUNG SEMARANG</t>
+  </si>
+  <si>
+    <t>(PKM) PENDAMPINGAN PEMBENAHAN INSTALASI JARINGAN INTERNET LPQ ANNUR TANGGUL MAS BARAT SEMARANG</t>
+  </si>
+  <si>
+    <t>PENDAMPINGAN PEMBENAHAN INSTALASI KELISTRIKAN GENSET PANTI ASUHAN SULTAN FATAH NGALIYAN SEMARANG</t>
+  </si>
+  <si>
+    <t>SOSIALISASI UMKM TERKAIT INOVASI LABEL PEYEK</t>
+  </si>
+  <si>
+    <t>PENDAMPINGAN PENCEGAHAN WASPADA DEMAM BERDARAH</t>
+  </si>
+  <si>
+    <t>PENDAMPINGAN PENGENALAN TEKNOLOGI INFORMASI DAN KOMUNIKASI DALAM PEMASANG WIFI SETIAP WILAYAH KUPANG LOR AMBARAWA, KABUPATEN SEMARANG</t>
+  </si>
+  <si>
+    <t>Pemberdayaan Masyarakat Peternak Sapi Lokal Di Desa Kuripan Kecamatan Karangawen Kabupaten Demak Menuju Desa Sentra Energi Terbarukan</t>
+  </si>
+  <si>
+    <t>PELATIHAN MADING DIGITAL BERBASIS WEB BAGI KOMUNITAS SENI HYSTERIA SEMARANG</t>
+  </si>
+  <si>
+    <t>PKM BAGI SD NEGERI KALIBANTENG KULON 01 SEMARANG</t>
+  </si>
+  <si>
+    <t>PENGUATAN PEMBUATAN MEDIA PEMBELAJARAN INTERAKTIF BERBASIS IT MGMP IPA BLORA</t>
+  </si>
+  <si>
+    <t>PENGUATAN PEMBUATAN MEDIA PEMBELAJARAN INTERAKTIF BERBASIS IT MGMP IPA GROBOGAN</t>
+  </si>
+  <si>
+    <t>PKM MODEL PEMBELAJARAN BERBASIS DIGITAL BAGI GURU-GURU SMPN 3 SEMARANG</t>
+  </si>
+  <si>
+    <t>MEMBUAT MEDIA UNTUK POJOK BACA DI KABUPATEN KENDAL</t>
+  </si>
+  <si>
+    <t>PENGEDUKASIAN TERHADAP WARGA DESA LIMBANGAN, KENDAL UNTUK PEMANFAATAN LIMBAH ORGANIC MENJADI SABUN SERBA GUNA</t>
+  </si>
+  <si>
+    <t>PENGUATAN KARYA ILMIAH REMAJA (KIR) SISWA MAN 1 KOTA SEMARANG</t>
+  </si>
+  <si>
+    <t>PKM PENGUATAN PENYUSUNAN KARYA TULIS ILMIAH MGMP FISIKA KABUPATEN BOYOLALI</t>
+  </si>
+  <si>
+    <t>Bambang Hadi KunaryoGanjar Winasis; Afeef Kurnia Rahmawan;</t>
+  </si>
+  <si>
+    <t>Rizky Muliani Dwi Ujianti Setyoningsih Wibowo; Bambang Hadi Kunaryo;</t>
+  </si>
+  <si>
+    <t>Margono Imadudin Harjanto; Bambang Hadi Kunaryo;</t>
+  </si>
+  <si>
+    <t>Slamet Supriyadi Muhammad Amiruddin; Nur Aksin;</t>
+  </si>
+  <si>
+    <t>Margono Muhammad Amiruddin; Imadudin Harjanto;</t>
+  </si>
+  <si>
+    <t>Muhammad Amiruddin Personils : -</t>
+  </si>
+  <si>
+    <t>Muhammad AmiruddinPersonils : -</t>
+  </si>
+  <si>
+    <t>Achmad Buchori Suwarno Widodo; Siti Maisyaroh Bakti Pertiwi; Adhi Kusmantoro;</t>
+  </si>
+  <si>
+    <t>Theodora Indriati Wardani Adhi Kusmantoro; Irna Farikhah;</t>
+  </si>
+  <si>
+    <t>Adhi Kusmantoro Irna Farikhah; Theodora Indriati Wardani;</t>
+  </si>
+  <si>
+    <t>Affandi Faisal Kurniawan REGULER ( PKM-REGULER )Nur Khoiri; Sigit Ristanto;</t>
+  </si>
+  <si>
+    <t>Affandi Faisal Kurniawan PROGRAM KEMITRAAN MAYSARAKAT-REGULER ( PKM-REGULER )Nur Khoiri; Sigit Ristanto;</t>
+  </si>
+  <si>
+    <t>Maria Yosephine Widarti Lestari PROGRAM KEMITRAAN MAYSARAKAT-REGULER ( PKM-REGULER )Sigit Ristanto; Jafar Sodiq;</t>
+  </si>
+  <si>
+    <t>Sigit Ristanto REGULER ( REG )Personils : -</t>
+  </si>
+  <si>
+    <t>Sigit Ristanto PROGRAM KEMITRAAN MASYARAKAT-REGULER ( PKM-REG )Nur Khoiri; Affandi Faisal Kurniawan;</t>
+  </si>
+  <si>
+    <t>Sigit Ristanto PROGRAM KEMITRAAN MAYSARAKAT-PENUGASAN ( PKM-PENUGASAN )Nur Khoiri; Affandi Faisal Kurniawan;</t>
+  </si>
+  <si>
+    <t>Rp8,000,000.00</t>
+  </si>
+  <si>
+    <t>Rp44,500,000.00</t>
+  </si>
+  <si>
+    <t>Rp1,320,000.00</t>
+  </si>
+  <si>
+    <t>Rp1,760,000.00</t>
+  </si>
+  <si>
+    <t>Rp101,121,000.00</t>
+  </si>
+  <si>
+    <t>Rp5,750,000.00</t>
+  </si>
+  <si>
+    <t>Rp6,000,000.00</t>
+  </si>
+  <si>
+    <t>Rp1,650,000.00</t>
+  </si>
+  <si>
+    <t>Rp1,430,000.00</t>
+  </si>
+  <si>
+    <t>Rp14,000,000.00</t>
+  </si>
+  <si>
+    <t> REGULER ( PKM-REGULER )</t>
+  </si>
+  <si>
+    <t>KOMPETITIF NASIONAL ( PKM )</t>
+  </si>
+  <si>
+    <t>PROGRAM KEMITRAAN MASYARAKAT ( PKM )</t>
+  </si>
+  <si>
+    <t>MANDIRI ( PKM-MANDIRI )</t>
+  </si>
+  <si>
+    <t>PROGRAM KEMITRAAN MAYSARAKAT-REGULER ( PKM-REGULER )</t>
+  </si>
+  <si>
+    <t>REGULER ( REG )</t>
+  </si>
+  <si>
+    <t>Pengabdian Kepada Masyarakat Kompetitif Nasional ( PDB )</t>
   </si>
 </sst>
 </file>
@@ -1688,8 +2103,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2032,81 +2451,81 @@
         <v>110</v>
       </c>
       <c r="B1" t="s">
-        <v>380</v>
+        <v>343</v>
       </c>
       <c r="C1" t="s">
-        <v>381</v>
+        <v>344</v>
       </c>
       <c r="D1" t="s">
-        <v>382</v>
+        <v>345</v>
       </c>
       <c r="E1" t="s">
-        <v>383</v>
+        <v>346</v>
       </c>
       <c r="F1" t="s">
-        <v>384</v>
+        <v>347</v>
       </c>
       <c r="G1" t="s">
-        <v>385</v>
+        <v>348</v>
       </c>
       <c r="H1" t="s">
-        <v>386</v>
+        <v>349</v>
       </c>
       <c r="I1" t="s">
-        <v>387</v>
+        <v>350</v>
       </c>
       <c r="J1" t="s">
-        <v>388</v>
+        <v>351</v>
       </c>
       <c r="K1" t="s">
-        <v>389</v>
+        <v>352</v>
       </c>
       <c r="L1" t="s">
-        <v>390</v>
+        <v>353</v>
       </c>
       <c r="M1" t="s">
-        <v>391</v>
+        <v>354</v>
       </c>
       <c r="N1" t="s">
-        <v>392</v>
+        <v>355</v>
       </c>
       <c r="O1" t="s">
-        <v>393</v>
+        <v>356</v>
       </c>
       <c r="P1" t="s">
-        <v>394</v>
+        <v>357</v>
       </c>
       <c r="Q1" t="s">
-        <v>395</v>
+        <v>358</v>
       </c>
       <c r="R1" t="s">
-        <v>396</v>
+        <v>359</v>
       </c>
       <c r="S1" t="s">
-        <v>397</v>
+        <v>360</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>398</v>
+        <v>361</v>
       </c>
       <c r="B2" t="s">
-        <v>399</v>
+        <v>362</v>
       </c>
       <c r="C2" t="s">
-        <v>400</v>
+        <v>363</v>
       </c>
       <c r="D2" t="s">
-        <v>401</v>
+        <v>364</v>
       </c>
       <c r="E2" t="s">
-        <v>402</v>
+        <v>365</v>
       </c>
       <c r="F2" t="s">
-        <v>403</v>
+        <v>366</v>
       </c>
       <c r="G2" t="s">
-        <v>404</v>
+        <v>367</v>
       </c>
       <c r="H2">
         <v>203</v>
@@ -2115,34 +2534,34 @@
         <v>3.32</v>
       </c>
       <c r="J2" t="s">
-        <v>405</v>
+        <v>368</v>
       </c>
       <c r="K2" t="s">
-        <v>406</v>
+        <v>369</v>
       </c>
       <c r="L2" t="s">
-        <v>407</v>
+        <v>370</v>
       </c>
       <c r="M2" t="s">
-        <v>408</v>
+        <v>371</v>
       </c>
       <c r="N2" t="s">
-        <v>409</v>
+        <v>372</v>
       </c>
       <c r="O2" t="s">
-        <v>410</v>
+        <v>373</v>
       </c>
       <c r="P2" t="s">
-        <v>411</v>
+        <v>374</v>
       </c>
       <c r="Q2" t="s">
-        <v>412</v>
+        <v>375</v>
       </c>
       <c r="R2" t="s">
-        <v>413</v>
+        <v>376</v>
       </c>
       <c r="S2" t="s">
-        <v>414</v>
+        <v>377</v>
       </c>
     </row>
   </sheetData>
@@ -2163,19 +2582,19 @@
         <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>317</v>
+        <v>297</v>
       </c>
       <c r="D1" t="s">
-        <v>282</v>
+        <v>262</v>
       </c>
       <c r="E1" t="s">
         <v>51</v>
       </c>
       <c r="F1" t="s">
-        <v>415</v>
+        <v>378</v>
       </c>
       <c r="G1" t="s">
-        <v>416</v>
+        <v>379</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
@@ -2183,22 +2602,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>417</v>
+        <v>380</v>
       </c>
       <c r="C2" t="s">
-        <v>418</v>
+        <v>381</v>
       </c>
       <c r="D2" t="s">
-        <v>419</v>
+        <v>382</v>
       </c>
       <c r="E2" t="s">
-        <v>420</v>
+        <v>383</v>
       </c>
       <c r="F2" t="s">
-        <v>421</v>
+        <v>384</v>
       </c>
       <c r="G2" t="s">
-        <v>422</v>
+        <v>385</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -2206,22 +2625,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>423</v>
+        <v>386</v>
       </c>
       <c r="C3" t="s">
-        <v>424</v>
+        <v>387</v>
       </c>
       <c r="D3" t="s">
-        <v>425</v>
+        <v>388</v>
       </c>
       <c r="E3" t="s">
-        <v>420</v>
+        <v>383</v>
       </c>
       <c r="F3" t="s">
-        <v>426</v>
+        <v>389</v>
       </c>
       <c r="G3" t="s">
-        <v>427</v>
+        <v>390</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -2229,22 +2648,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>428</v>
+        <v>391</v>
       </c>
       <c r="C4" t="s">
-        <v>429</v>
+        <v>392</v>
       </c>
       <c r="D4" t="s">
-        <v>430</v>
+        <v>393</v>
       </c>
       <c r="E4" t="s">
-        <v>431</v>
+        <v>394</v>
       </c>
       <c r="F4" t="s">
-        <v>432</v>
+        <v>395</v>
       </c>
       <c r="G4" t="s">
-        <v>433</v>
+        <v>396</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -2252,22 +2671,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>434</v>
+        <v>397</v>
       </c>
       <c r="C5" t="s">
-        <v>435</v>
+        <v>398</v>
       </c>
       <c r="D5" t="s">
-        <v>436</v>
+        <v>399</v>
       </c>
       <c r="E5" t="s">
-        <v>431</v>
+        <v>394</v>
       </c>
       <c r="F5" t="s">
-        <v>437</v>
+        <v>400</v>
       </c>
       <c r="G5" t="s">
-        <v>438</v>
+        <v>401</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -2275,22 +2694,22 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>439</v>
+        <v>402</v>
       </c>
       <c r="C6" t="s">
-        <v>440</v>
+        <v>403</v>
       </c>
       <c r="D6" t="s">
-        <v>419</v>
+        <v>382</v>
       </c>
       <c r="E6" t="s">
-        <v>431</v>
+        <v>394</v>
       </c>
       <c r="F6" t="s">
-        <v>441</v>
+        <v>404</v>
       </c>
       <c r="G6" t="s">
-        <v>442</v>
+        <v>405</v>
       </c>
     </row>
   </sheetData>
@@ -2308,31 +2727,31 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>443</v>
+        <v>406</v>
       </c>
       <c r="C1" t="s">
-        <v>444</v>
+        <v>407</v>
       </c>
       <c r="D1" t="s">
-        <v>445</v>
+        <v>408</v>
       </c>
       <c r="E1" t="s">
-        <v>446</v>
+        <v>409</v>
       </c>
       <c r="F1" t="s">
-        <v>447</v>
+        <v>410</v>
       </c>
       <c r="G1" t="s">
         <v>12</v>
       </c>
       <c r="H1" t="s">
-        <v>448</v>
+        <v>411</v>
       </c>
       <c r="I1" t="s">
-        <v>449</v>
+        <v>412</v>
       </c>
       <c r="J1" t="s">
-        <v>450</v>
+        <v>413</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -2340,31 +2759,31 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>451</v>
+        <v>414</v>
       </c>
       <c r="C2" t="s">
-        <v>452</v>
+        <v>415</v>
       </c>
       <c r="D2" t="s">
-        <v>453</v>
+        <v>416</v>
       </c>
       <c r="E2" t="s">
-        <v>454</v>
+        <v>417</v>
       </c>
       <c r="F2" t="s">
-        <v>455</v>
+        <v>418</v>
       </c>
       <c r="G2" t="s">
-        <v>456</v>
+        <v>419</v>
       </c>
       <c r="H2" t="s">
-        <v>457</v>
+        <v>420</v>
       </c>
       <c r="I2" t="s">
-        <v>458</v>
+        <v>421</v>
       </c>
       <c r="J2" t="s">
-        <v>459</v>
+        <v>422</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
@@ -2372,31 +2791,31 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>460</v>
+        <v>423</v>
       </c>
       <c r="C3" t="s">
-        <v>452</v>
+        <v>415</v>
       </c>
       <c r="D3" t="s">
-        <v>461</v>
+        <v>424</v>
       </c>
       <c r="E3" t="s">
-        <v>462</v>
+        <v>425</v>
       </c>
       <c r="F3" t="s">
-        <v>463</v>
+        <v>426</v>
       </c>
       <c r="G3" t="s">
-        <v>464</v>
+        <v>427</v>
       </c>
       <c r="H3" t="s">
-        <v>465</v>
+        <v>428</v>
       </c>
       <c r="I3" t="s">
-        <v>466</v>
+        <v>429</v>
       </c>
       <c r="J3" t="s">
-        <v>467</v>
+        <v>430</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -2404,31 +2823,31 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>468</v>
+        <v>431</v>
       </c>
       <c r="C4" t="s">
-        <v>469</v>
+        <v>432</v>
       </c>
       <c r="D4" t="s">
-        <v>470</v>
+        <v>433</v>
       </c>
       <c r="E4" t="s">
-        <v>471</v>
+        <v>434</v>
       </c>
       <c r="F4" t="s">
-        <v>472</v>
+        <v>435</v>
       </c>
       <c r="G4" t="s">
-        <v>473</v>
+        <v>436</v>
       </c>
       <c r="H4" t="s">
-        <v>474</v>
+        <v>437</v>
       </c>
       <c r="I4" t="s">
-        <v>475</v>
+        <v>438</v>
       </c>
       <c r="J4" t="s">
-        <v>476</v>
+        <v>439</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -2436,31 +2855,31 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>477</v>
+        <v>440</v>
       </c>
       <c r="C5" t="s">
-        <v>478</v>
+        <v>441</v>
       </c>
       <c r="D5" t="s">
-        <v>479</v>
+        <v>442</v>
       </c>
       <c r="E5" t="s">
-        <v>480</v>
+        <v>443</v>
       </c>
       <c r="F5" t="s">
-        <v>481</v>
+        <v>444</v>
       </c>
       <c r="G5" t="s">
-        <v>482</v>
+        <v>445</v>
       </c>
       <c r="H5" t="s">
-        <v>483</v>
+        <v>446</v>
       </c>
       <c r="I5" t="s">
-        <v>484</v>
+        <v>447</v>
       </c>
       <c r="J5" t="s">
-        <v>485</v>
+        <v>448</v>
       </c>
     </row>
   </sheetData>
@@ -2481,7 +2900,7 @@
         <v>110</v>
       </c>
       <c r="C1" t="s">
-        <v>486</v>
+        <v>449</v>
       </c>
       <c r="D1" t="s">
         <v>8</v>
@@ -2490,7 +2909,7 @@
         <v>51</v>
       </c>
       <c r="F1" t="s">
-        <v>487</v>
+        <v>450</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -2498,19 +2917,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>488</v>
+        <v>451</v>
       </c>
       <c r="C2" t="s">
-        <v>489</v>
+        <v>452</v>
       </c>
       <c r="D2" t="s">
-        <v>490</v>
+        <v>453</v>
       </c>
       <c r="E2" t="s">
-        <v>431</v>
+        <v>394</v>
       </c>
       <c r="F2" t="s">
-        <v>491</v>
+        <v>454</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -2518,19 +2937,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>492</v>
+        <v>455</v>
       </c>
       <c r="C3" t="s">
-        <v>493</v>
+        <v>456</v>
       </c>
       <c r="D3" t="s">
-        <v>494</v>
+        <v>457</v>
       </c>
       <c r="E3" t="s">
-        <v>431</v>
+        <v>394</v>
       </c>
       <c r="F3" t="s">
-        <v>495</v>
+        <v>458</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -2538,19 +2957,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>496</v>
+        <v>459</v>
       </c>
       <c r="C4" t="s">
-        <v>497</v>
+        <v>460</v>
       </c>
       <c r="D4" t="s">
-        <v>494</v>
+        <v>457</v>
       </c>
       <c r="E4" t="s">
-        <v>431</v>
+        <v>394</v>
       </c>
       <c r="F4" t="s">
-        <v>498</v>
+        <v>461</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -2558,19 +2977,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>499</v>
+        <v>462</v>
       </c>
       <c r="C5" t="s">
-        <v>500</v>
+        <v>463</v>
       </c>
       <c r="D5" t="s">
-        <v>494</v>
+        <v>457</v>
       </c>
       <c r="E5" t="s">
-        <v>431</v>
+        <v>394</v>
       </c>
       <c r="F5" t="s">
-        <v>501</v>
+        <v>464</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -2578,19 +2997,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>502</v>
+        <v>465</v>
       </c>
       <c r="C6" t="s">
-        <v>503</v>
+        <v>466</v>
       </c>
       <c r="D6" t="s">
-        <v>504</v>
+        <v>467</v>
       </c>
       <c r="E6" t="s">
-        <v>431</v>
+        <v>394</v>
       </c>
       <c r="F6" t="s">
-        <v>505</v>
+        <v>468</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -2598,19 +3017,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>506</v>
+        <v>469</v>
       </c>
       <c r="C7" t="s">
-        <v>507</v>
+        <v>470</v>
       </c>
       <c r="D7" t="s">
-        <v>504</v>
+        <v>467</v>
       </c>
       <c r="E7" t="s">
-        <v>431</v>
+        <v>394</v>
       </c>
       <c r="F7" t="s">
-        <v>508</v>
+        <v>471</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
@@ -2618,19 +3037,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>509</v>
+        <v>472</v>
       </c>
       <c r="C8" t="s">
-        <v>510</v>
+        <v>473</v>
       </c>
       <c r="D8" t="s">
-        <v>504</v>
+        <v>467</v>
       </c>
       <c r="E8" t="s">
-        <v>431</v>
+        <v>394</v>
       </c>
       <c r="F8" t="s">
-        <v>511</v>
+        <v>474</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
@@ -2638,19 +3057,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>512</v>
+        <v>475</v>
       </c>
       <c r="C9" t="s">
-        <v>513</v>
+        <v>476</v>
       </c>
       <c r="D9" t="s">
-        <v>514</v>
+        <v>477</v>
       </c>
       <c r="E9" t="s">
-        <v>431</v>
+        <v>394</v>
       </c>
       <c r="F9" t="s">
-        <v>515</v>
+        <v>478</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
@@ -2658,19 +3077,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>516</v>
+        <v>479</v>
       </c>
       <c r="C10" t="s">
-        <v>517</v>
+        <v>480</v>
       </c>
       <c r="D10" t="s">
-        <v>514</v>
+        <v>477</v>
       </c>
       <c r="E10" t="s">
-        <v>431</v>
+        <v>394</v>
       </c>
       <c r="F10" t="s">
-        <v>518</v>
+        <v>481</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
@@ -2678,19 +3097,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>519</v>
+        <v>482</v>
       </c>
       <c r="C11" t="s">
-        <v>520</v>
+        <v>483</v>
       </c>
       <c r="D11" t="s">
-        <v>521</v>
+        <v>484</v>
       </c>
       <c r="E11" t="s">
-        <v>431</v>
+        <v>394</v>
       </c>
       <c r="F11" t="s">
-        <v>522</v>
+        <v>485</v>
       </c>
     </row>
   </sheetData>
@@ -3187,6 +3606,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="32.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.35">
@@ -3232,34 +3652,34 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>523</v>
+        <v>486</v>
       </c>
       <c r="C2" t="s">
-        <v>531</v>
+        <v>494</v>
       </c>
       <c r="D2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E2" t="s">
         <v>121</v>
       </c>
       <c r="F2" t="s">
+        <v>502</v>
+      </c>
+      <c r="G2" t="s">
+        <v>509</v>
+      </c>
+      <c r="H2" t="s">
         <v>122</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>123</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>124</v>
       </c>
-      <c r="I2" t="s">
+      <c r="L2" t="s">
         <v>125</v>
-      </c>
-      <c r="J2" t="s">
-        <v>126</v>
-      </c>
-      <c r="L2" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
@@ -3267,34 +3687,34 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>524</v>
+        <v>487</v>
       </c>
       <c r="C3" t="s">
-        <v>532</v>
+        <v>495</v>
       </c>
       <c r="D3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E3" t="s">
+        <v>128</v>
+      </c>
+      <c r="F3" t="s">
+        <v>502</v>
+      </c>
+      <c r="G3" t="s">
+        <v>510</v>
+      </c>
+      <c r="H3" t="s">
+        <v>515</v>
+      </c>
+      <c r="I3" t="s">
         <v>129</v>
       </c>
-      <c r="E3" t="s">
+      <c r="J3" t="s">
         <v>130</v>
       </c>
-      <c r="F3" t="s">
-        <v>131</v>
-      </c>
-      <c r="G3" t="s">
-        <v>132</v>
-      </c>
-      <c r="H3" t="s">
-        <v>133</v>
-      </c>
-      <c r="I3" t="s">
-        <v>134</v>
-      </c>
-      <c r="J3" t="s">
-        <v>135</v>
-      </c>
       <c r="L3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
@@ -3302,34 +3722,31 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>525</v>
+        <v>488</v>
       </c>
       <c r="C4" t="s">
-        <v>533</v>
+        <v>496</v>
       </c>
       <c r="D4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E4" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="F4" t="s">
-        <v>137</v>
-      </c>
-      <c r="G4" t="s">
-        <v>138</v>
+        <v>503</v>
       </c>
       <c r="H4" t="s">
-        <v>139</v>
+        <v>516</v>
       </c>
       <c r="I4" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="J4" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="L4" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
@@ -3337,34 +3754,34 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>526</v>
+        <v>489</v>
       </c>
       <c r="C5" t="s">
-        <v>534</v>
+        <v>497</v>
       </c>
       <c r="D5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E5" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="F5" t="s">
-        <v>143</v>
+        <v>504</v>
       </c>
       <c r="G5" t="s">
-        <v>144</v>
+        <v>511</v>
       </c>
       <c r="H5" t="s">
-        <v>145</v>
+        <v>516</v>
       </c>
       <c r="I5" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="J5" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="L5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
@@ -3372,34 +3789,34 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>527</v>
+        <v>490</v>
       </c>
       <c r="C6" t="s">
-        <v>535</v>
+        <v>498</v>
       </c>
       <c r="D6" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="E6" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="F6" t="s">
-        <v>150</v>
+        <v>505</v>
       </c>
       <c r="G6" t="s">
-        <v>151</v>
+        <v>512</v>
       </c>
       <c r="H6" t="s">
-        <v>152</v>
+        <v>139</v>
       </c>
       <c r="I6" t="s">
-        <v>153</v>
+        <v>140</v>
       </c>
       <c r="J6" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="L6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
@@ -3407,34 +3824,31 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>528</v>
+        <v>491</v>
       </c>
       <c r="C7" t="s">
-        <v>536</v>
+        <v>499</v>
       </c>
       <c r="D7" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="E7" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="F7" t="s">
-        <v>156</v>
+        <v>506</v>
       </c>
       <c r="G7" t="s">
-        <v>157</v>
-      </c>
-      <c r="H7" t="s">
-        <v>158</v>
+        <v>508</v>
       </c>
       <c r="I7" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="J7" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="L7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
@@ -3442,34 +3856,31 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>529</v>
+        <v>492</v>
       </c>
       <c r="C8" t="s">
-        <v>537</v>
+        <v>500</v>
       </c>
       <c r="D8" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E8" t="s">
-        <v>161</v>
-      </c>
-      <c r="F8" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="G8" t="s">
-        <v>162</v>
+        <v>513</v>
       </c>
       <c r="H8" t="s">
-        <v>163</v>
+        <v>139</v>
       </c>
       <c r="I8" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
       <c r="J8" t="s">
-        <v>165</v>
+        <v>147</v>
       </c>
       <c r="L8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
@@ -3477,34 +3888,31 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>530</v>
+        <v>493</v>
       </c>
       <c r="C9" t="s">
-        <v>538</v>
+        <v>501</v>
       </c>
       <c r="D9" t="s">
         <v>120</v>
       </c>
       <c r="E9" t="s">
-        <v>166</v>
+        <v>148</v>
       </c>
       <c r="F9" t="s">
-        <v>143</v>
+        <v>507</v>
       </c>
       <c r="G9" t="s">
-        <v>167</v>
-      </c>
-      <c r="H9" t="s">
-        <v>168</v>
+        <v>514</v>
       </c>
       <c r="I9" t="s">
-        <v>169</v>
+        <v>149</v>
       </c>
       <c r="J9" t="s">
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="L9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -3522,22 +3930,22 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>171</v>
+        <v>151</v>
       </c>
       <c r="C1" t="s">
         <v>110</v>
       </c>
       <c r="D1" t="s">
-        <v>172</v>
+        <v>152</v>
       </c>
       <c r="E1" t="s">
-        <v>173</v>
+        <v>153</v>
       </c>
       <c r="F1" t="s">
-        <v>174</v>
+        <v>154</v>
       </c>
       <c r="G1" t="s">
-        <v>175</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
@@ -3545,10 +3953,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>176</v>
+        <v>156</v>
       </c>
       <c r="C2" t="s">
-        <v>177</v>
+        <v>157</v>
       </c>
       <c r="D2">
         <v>3</v>
@@ -3557,10 +3965,10 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
       <c r="G2" t="s">
-        <v>179</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -3568,10 +3976,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="C3" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D3">
         <v>3</v>
@@ -3580,10 +3988,10 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
       <c r="G3" t="s">
-        <v>182</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -3591,10 +3999,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
       <c r="C4" t="s">
-        <v>184</v>
+        <v>164</v>
       </c>
       <c r="D4">
         <v>3</v>
@@ -3603,10 +4011,10 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G4" t="s">
-        <v>186</v>
+        <v>166</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -3614,10 +4022,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>187</v>
+        <v>167</v>
       </c>
       <c r="C5" t="s">
-        <v>188</v>
+        <v>168</v>
       </c>
       <c r="D5">
         <v>2</v>
@@ -3626,7 +4034,7 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -3634,10 +4042,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>189</v>
+        <v>169</v>
       </c>
       <c r="C6" t="s">
-        <v>190</v>
+        <v>170</v>
       </c>
       <c r="D6">
         <v>2</v>
@@ -3646,10 +4054,10 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
       <c r="G6" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -3657,10 +4065,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="C7" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="D7">
         <v>2</v>
@@ -3669,10 +4077,10 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
       <c r="G7" t="s">
-        <v>194</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
@@ -3680,10 +4088,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="C8" t="s">
-        <v>196</v>
+        <v>176</v>
       </c>
       <c r="D8">
         <v>3</v>
@@ -3692,10 +4100,10 @@
         <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
       <c r="G8" t="s">
-        <v>197</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -3703,10 +4111,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>198</v>
+        <v>178</v>
       </c>
       <c r="C9" t="s">
-        <v>199</v>
+        <v>179</v>
       </c>
       <c r="D9">
         <v>3</v>
@@ -3715,10 +4123,10 @@
         <v>2</v>
       </c>
       <c r="F9" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G9" t="s">
-        <v>200</v>
+        <v>180</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
@@ -3726,10 +4134,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>201</v>
+        <v>181</v>
       </c>
       <c r="C10" t="s">
-        <v>202</v>
+        <v>182</v>
       </c>
       <c r="D10">
         <v>3</v>
@@ -3738,10 +4146,10 @@
         <v>2</v>
       </c>
       <c r="F10" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G10" t="s">
-        <v>203</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -3749,10 +4157,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>204</v>
+        <v>184</v>
       </c>
       <c r="C11" t="s">
-        <v>205</v>
+        <v>185</v>
       </c>
       <c r="D11">
         <v>3</v>
@@ -3761,10 +4169,10 @@
         <v>2</v>
       </c>
       <c r="F11" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
       <c r="G11" t="s">
-        <v>206</v>
+        <v>186</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
@@ -3772,10 +4180,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>207</v>
+        <v>187</v>
       </c>
       <c r="C12" t="s">
-        <v>208</v>
+        <v>188</v>
       </c>
       <c r="D12">
         <v>2</v>
@@ -3784,7 +4192,7 @@
         <v>2</v>
       </c>
       <c r="F12" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
@@ -3792,10 +4200,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>209</v>
+        <v>189</v>
       </c>
       <c r="C13" t="s">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="D13">
         <v>3</v>
@@ -3804,10 +4212,10 @@
         <v>3</v>
       </c>
       <c r="F13" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G13" t="s">
-        <v>211</v>
+        <v>191</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
@@ -3815,10 +4223,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>212</v>
+        <v>192</v>
       </c>
       <c r="C14" t="s">
-        <v>213</v>
+        <v>193</v>
       </c>
       <c r="D14">
         <v>3</v>
@@ -3827,10 +4235,10 @@
         <v>3</v>
       </c>
       <c r="F14" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G14" t="s">
-        <v>214</v>
+        <v>194</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
@@ -3838,10 +4246,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>215</v>
+        <v>195</v>
       </c>
       <c r="C15" t="s">
-        <v>216</v>
+        <v>196</v>
       </c>
       <c r="D15">
         <v>3</v>
@@ -3850,10 +4258,10 @@
         <v>3</v>
       </c>
       <c r="F15" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G15" t="s">
-        <v>217</v>
+        <v>197</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
@@ -3861,10 +4269,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>218</v>
+        <v>198</v>
       </c>
       <c r="C16" t="s">
-        <v>219</v>
+        <v>199</v>
       </c>
       <c r="D16">
         <v>3</v>
@@ -3873,10 +4281,10 @@
         <v>3</v>
       </c>
       <c r="F16" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G16" t="s">
-        <v>220</v>
+        <v>200</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
@@ -3884,10 +4292,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>221</v>
+        <v>201</v>
       </c>
       <c r="C17" t="s">
-        <v>222</v>
+        <v>202</v>
       </c>
       <c r="D17">
         <v>3</v>
@@ -3896,10 +4304,10 @@
         <v>3</v>
       </c>
       <c r="F17" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G17" t="s">
-        <v>223</v>
+        <v>203</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
@@ -3907,10 +4315,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>224</v>
+        <v>204</v>
       </c>
       <c r="C18" t="s">
-        <v>225</v>
+        <v>205</v>
       </c>
       <c r="D18">
         <v>3</v>
@@ -3919,10 +4327,10 @@
         <v>4</v>
       </c>
       <c r="F18" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G18" t="s">
-        <v>226</v>
+        <v>206</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -3930,10 +4338,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>227</v>
+        <v>207</v>
       </c>
       <c r="C19" t="s">
-        <v>228</v>
+        <v>208</v>
       </c>
       <c r="D19">
         <v>3</v>
@@ -3942,10 +4350,10 @@
         <v>4</v>
       </c>
       <c r="F19" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G19" t="s">
-        <v>229</v>
+        <v>209</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
@@ -3953,10 +4361,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>230</v>
+        <v>210</v>
       </c>
       <c r="C20" t="s">
-        <v>231</v>
+        <v>211</v>
       </c>
       <c r="D20">
         <v>3</v>
@@ -3965,10 +4373,10 @@
         <v>4</v>
       </c>
       <c r="F20" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G20" t="s">
-        <v>232</v>
+        <v>212</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -3976,10 +4384,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>233</v>
+        <v>213</v>
       </c>
       <c r="C21" t="s">
-        <v>234</v>
+        <v>214</v>
       </c>
       <c r="D21">
         <v>3</v>
@@ -3988,10 +4396,10 @@
         <v>4</v>
       </c>
       <c r="F21" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G21" t="s">
-        <v>235</v>
+        <v>215</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
@@ -3999,10 +4407,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>236</v>
+        <v>216</v>
       </c>
       <c r="C22" t="s">
-        <v>237</v>
+        <v>217</v>
       </c>
       <c r="D22">
         <v>3</v>
@@ -4011,7 +4419,7 @@
         <v>4</v>
       </c>
       <c r="F22" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
@@ -4019,10 +4427,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>238</v>
+        <v>218</v>
       </c>
       <c r="C23" t="s">
-        <v>239</v>
+        <v>219</v>
       </c>
       <c r="D23">
         <v>3</v>
@@ -4031,10 +4439,10 @@
         <v>5</v>
       </c>
       <c r="F23" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G23" t="s">
-        <v>240</v>
+        <v>220</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
@@ -4042,10 +4450,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>241</v>
+        <v>221</v>
       </c>
       <c r="C24" t="s">
-        <v>242</v>
+        <v>222</v>
       </c>
       <c r="D24">
         <v>3</v>
@@ -4054,10 +4462,10 @@
         <v>5</v>
       </c>
       <c r="F24" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G24" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
@@ -4065,10 +4473,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>244</v>
+        <v>224</v>
       </c>
       <c r="C25" t="s">
-        <v>245</v>
+        <v>225</v>
       </c>
       <c r="D25">
         <v>3</v>
@@ -4077,10 +4485,10 @@
         <v>5</v>
       </c>
       <c r="F25" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G25" t="s">
-        <v>246</v>
+        <v>226</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
@@ -4088,10 +4496,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>247</v>
+        <v>227</v>
       </c>
       <c r="C26" t="s">
-        <v>248</v>
+        <v>228</v>
       </c>
       <c r="D26">
         <v>3</v>
@@ -4100,10 +4508,10 @@
         <v>5</v>
       </c>
       <c r="F26" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G26" t="s">
-        <v>249</v>
+        <v>229</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
@@ -4111,10 +4519,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="C27" t="s">
-        <v>251</v>
+        <v>231</v>
       </c>
       <c r="D27">
         <v>2</v>
@@ -4123,7 +4531,7 @@
         <v>5</v>
       </c>
       <c r="F27" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
@@ -4131,10 +4539,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>252</v>
+        <v>232</v>
       </c>
       <c r="C28" t="s">
-        <v>253</v>
+        <v>233</v>
       </c>
       <c r="D28">
         <v>3</v>
@@ -4143,10 +4551,10 @@
         <v>6</v>
       </c>
       <c r="F28" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G28" t="s">
-        <v>254</v>
+        <v>234</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
@@ -4154,10 +4562,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>255</v>
+        <v>235</v>
       </c>
       <c r="C29" t="s">
-        <v>256</v>
+        <v>236</v>
       </c>
       <c r="D29">
         <v>3</v>
@@ -4166,10 +4574,10 @@
         <v>6</v>
       </c>
       <c r="F29" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G29" t="s">
-        <v>257</v>
+        <v>237</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
@@ -4177,10 +4585,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>258</v>
+        <v>238</v>
       </c>
       <c r="C30" t="s">
-        <v>259</v>
+        <v>239</v>
       </c>
       <c r="D30">
         <v>3</v>
@@ -4189,10 +4597,10 @@
         <v>6</v>
       </c>
       <c r="F30" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G30" t="s">
-        <v>260</v>
+        <v>240</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
@@ -4200,10 +4608,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>261</v>
+        <v>241</v>
       </c>
       <c r="C31" t="s">
-        <v>262</v>
+        <v>242</v>
       </c>
       <c r="D31">
         <v>2</v>
@@ -4212,7 +4620,7 @@
         <v>6</v>
       </c>
       <c r="F31" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
@@ -4220,10 +4628,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C32" t="s">
-        <v>264</v>
+        <v>244</v>
       </c>
       <c r="D32">
         <v>2</v>
@@ -4232,10 +4640,10 @@
         <v>6</v>
       </c>
       <c r="F32" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
       <c r="G32" t="s">
-        <v>265</v>
+        <v>245</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
@@ -4243,10 +4651,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>266</v>
+        <v>246</v>
       </c>
       <c r="C33" t="s">
-        <v>267</v>
+        <v>247</v>
       </c>
       <c r="D33">
         <v>3</v>
@@ -4255,10 +4663,10 @@
         <v>7</v>
       </c>
       <c r="F33" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G33" t="s">
-        <v>268</v>
+        <v>248</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
@@ -4266,10 +4674,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>269</v>
+        <v>249</v>
       </c>
       <c r="C34" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="D34">
         <v>3</v>
@@ -4278,10 +4686,10 @@
         <v>7</v>
       </c>
       <c r="F34" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G34" t="s">
-        <v>271</v>
+        <v>251</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
@@ -4289,10 +4697,10 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>272</v>
+        <v>252</v>
       </c>
       <c r="C35" t="s">
-        <v>273</v>
+        <v>253</v>
       </c>
       <c r="D35">
         <v>3</v>
@@ -4301,10 +4709,10 @@
         <v>7</v>
       </c>
       <c r="F35" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G35" t="s">
-        <v>274</v>
+        <v>254</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
@@ -4312,10 +4720,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>275</v>
+        <v>255</v>
       </c>
       <c r="C36" t="s">
-        <v>276</v>
+        <v>256</v>
       </c>
       <c r="D36">
         <v>2</v>
@@ -4324,7 +4732,7 @@
         <v>7</v>
       </c>
       <c r="F36" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
@@ -4332,10 +4740,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>277</v>
+        <v>257</v>
       </c>
       <c r="C37" t="s">
-        <v>278</v>
+        <v>258</v>
       </c>
       <c r="D37">
         <v>4</v>
@@ -4344,10 +4752,10 @@
         <v>8</v>
       </c>
       <c r="F37" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="G37" t="s">
-        <v>279</v>
+        <v>259</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
@@ -4355,10 +4763,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="C38" t="s">
-        <v>281</v>
+        <v>261</v>
       </c>
       <c r="D38">
         <v>6</v>
@@ -4367,7 +4775,7 @@
         <v>8</v>
       </c>
       <c r="F38" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -4388,13 +4796,13 @@
         <v>110</v>
       </c>
       <c r="C1" t="s">
-        <v>282</v>
+        <v>262</v>
       </c>
       <c r="D1" t="s">
         <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>283</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -4402,16 +4810,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>284</v>
+        <v>264</v>
       </c>
       <c r="C2" t="s">
-        <v>285</v>
+        <v>265</v>
       </c>
       <c r="D2" t="s">
-        <v>286</v>
+        <v>266</v>
       </c>
       <c r="E2" t="s">
-        <v>287</v>
+        <v>267</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -4419,16 +4827,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>288</v>
+        <v>268</v>
       </c>
       <c r="C3" t="s">
-        <v>289</v>
+        <v>269</v>
       </c>
       <c r="D3" t="s">
-        <v>290</v>
+        <v>270</v>
       </c>
       <c r="E3" t="s">
-        <v>291</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -4436,16 +4844,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>292</v>
+        <v>272</v>
       </c>
       <c r="C4" t="s">
-        <v>289</v>
+        <v>269</v>
       </c>
       <c r="D4" t="s">
-        <v>293</v>
+        <v>273</v>
       </c>
       <c r="E4" t="s">
-        <v>291</v>
+        <v>271</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -4453,16 +4861,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>294</v>
+        <v>274</v>
       </c>
       <c r="C5" t="s">
-        <v>295</v>
+        <v>275</v>
       </c>
       <c r="D5" t="s">
-        <v>296</v>
+        <v>276</v>
       </c>
       <c r="E5" t="s">
-        <v>297</v>
+        <v>277</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -4470,16 +4878,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>298</v>
+        <v>278</v>
       </c>
       <c r="C6" t="s">
         <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>299</v>
+        <v>279</v>
       </c>
       <c r="E6" t="s">
-        <v>291</v>
+        <v>271</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -4487,16 +4895,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>300</v>
+        <v>280</v>
       </c>
       <c r="C7" t="s">
-        <v>285</v>
+        <v>265</v>
       </c>
       <c r="D7" t="s">
-        <v>301</v>
+        <v>281</v>
       </c>
       <c r="E7" t="s">
-        <v>287</v>
+        <v>267</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -4504,16 +4912,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>302</v>
+        <v>282</v>
       </c>
       <c r="C8" t="s">
-        <v>303</v>
+        <v>283</v>
       </c>
       <c r="D8" t="s">
-        <v>304</v>
+        <v>284</v>
       </c>
       <c r="E8" t="s">
-        <v>287</v>
+        <v>267</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -4521,16 +4929,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>305</v>
+        <v>285</v>
       </c>
       <c r="C9" t="s">
-        <v>306</v>
+        <v>286</v>
       </c>
       <c r="D9" t="s">
-        <v>307</v>
+        <v>287</v>
       </c>
       <c r="E9" t="s">
-        <v>297</v>
+        <v>277</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -4538,16 +4946,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>308</v>
+        <v>288</v>
       </c>
       <c r="C10" t="s">
+        <v>269</v>
+      </c>
+      <c r="D10" t="s">
         <v>289</v>
       </c>
-      <c r="D10" t="s">
-        <v>309</v>
-      </c>
       <c r="E10" t="s">
-        <v>291</v>
+        <v>271</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -4555,16 +4963,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>310</v>
+        <v>290</v>
       </c>
       <c r="C11" t="s">
-        <v>303</v>
+        <v>283</v>
       </c>
       <c r="D11" t="s">
-        <v>311</v>
+        <v>291</v>
       </c>
       <c r="E11" t="s">
-        <v>297</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -4572,16 +4980,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="C12" t="s">
-        <v>313</v>
+        <v>293</v>
       </c>
       <c r="D12" t="s">
-        <v>314</v>
+        <v>294</v>
       </c>
       <c r="E12" t="s">
-        <v>291</v>
+        <v>271</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -4589,16 +4997,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>315</v>
+        <v>295</v>
       </c>
       <c r="C13" t="s">
-        <v>313</v>
+        <v>293</v>
       </c>
       <c r="D13" t="s">
-        <v>316</v>
+        <v>296</v>
       </c>
       <c r="E13" t="s">
-        <v>287</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -4608,33 +5016,37 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="8.7265625" style="2"/>
+    <col min="6" max="6" width="15.54296875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>317</v>
+        <v>297</v>
       </c>
       <c r="D1" t="s">
         <v>51</v>
       </c>
       <c r="E1" t="s">
-        <v>282</v>
+        <v>262</v>
       </c>
       <c r="F1" t="s">
-        <v>318</v>
+        <v>298</v>
       </c>
       <c r="G1" t="s">
-        <v>319</v>
+        <v>299</v>
       </c>
       <c r="H1" t="s">
-        <v>320</v>
+        <v>300</v>
       </c>
       <c r="I1" t="s">
         <v>12</v>
@@ -4647,119 +5059,1033 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>321</v>
+      <c r="B2" s="2" t="s">
+        <v>517</v>
       </c>
       <c r="C2" t="s">
-        <v>322</v>
+        <v>552</v>
       </c>
       <c r="D2" t="s">
-        <v>323</v>
+        <v>584</v>
       </c>
       <c r="E2" t="s">
         <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>324</v>
+        <v>589</v>
       </c>
       <c r="G2" t="s">
-        <v>325</v>
-      </c>
-      <c r="H2" t="s">
-        <v>326</v>
-      </c>
-      <c r="I2" t="s">
-        <v>327</v>
-      </c>
-      <c r="J2" t="s">
-        <v>328</v>
+        <v>605</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>329</v>
+      <c r="B3" s="2" t="s">
+        <v>518</v>
       </c>
       <c r="C3" t="s">
-        <v>128</v>
+        <v>553</v>
       </c>
       <c r="D3" t="s">
-        <v>323</v>
+        <v>584</v>
       </c>
       <c r="E3" t="s">
         <v>22</v>
       </c>
       <c r="F3" t="s">
-        <v>330</v>
+        <v>590</v>
       </c>
       <c r="G3" t="s">
-        <v>331</v>
-      </c>
-      <c r="H3" t="s">
-        <v>332</v>
-      </c>
-      <c r="I3" t="s">
-        <v>333</v>
+        <v>606</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>334</v>
+      <c r="B4" s="2" t="s">
+        <v>519</v>
       </c>
       <c r="C4" t="s">
-        <v>79</v>
+        <v>554</v>
       </c>
       <c r="D4" t="s">
-        <v>335</v>
+        <v>585</v>
       </c>
       <c r="E4" t="s">
         <v>22</v>
       </c>
-      <c r="F4" t="s">
-        <v>336</v>
-      </c>
       <c r="G4" t="s">
-        <v>325</v>
-      </c>
-      <c r="H4" t="s">
-        <v>161</v>
-      </c>
-      <c r="I4" t="s">
-        <v>337</v>
-      </c>
-      <c r="J4" t="s">
-        <v>338</v>
+        <v>605</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
-        <v>339</v>
+      <c r="B5" s="2" t="s">
+        <v>520</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>555</v>
       </c>
       <c r="D5" t="s">
-        <v>335</v>
+        <v>586</v>
       </c>
       <c r="E5" t="s">
         <v>22</v>
       </c>
-      <c r="F5" t="s">
-        <v>340</v>
-      </c>
       <c r="G5" t="s">
-        <v>331</v>
-      </c>
-      <c r="H5" t="s">
-        <v>341</v>
+        <v>605</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B6" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="C6" t="s">
+        <v>556</v>
+      </c>
+      <c r="D6" t="s">
+        <v>587</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>591</v>
+      </c>
+      <c r="G6" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B7" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="C7" t="s">
+        <v>557</v>
+      </c>
+      <c r="D7" t="s">
+        <v>584</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s">
+        <v>592</v>
+      </c>
+      <c r="G7" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B8" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="C8" t="s">
+        <v>558</v>
+      </c>
+      <c r="D8" t="s">
+        <v>586</v>
+      </c>
+      <c r="E8" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" t="s">
+        <v>593</v>
+      </c>
+      <c r="G8" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B9" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="C9" t="s">
+        <v>559</v>
+      </c>
+      <c r="D9" t="s">
+        <v>585</v>
+      </c>
+      <c r="E9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" t="s">
+        <v>594</v>
+      </c>
+      <c r="G9" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B10" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="C10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D10" t="s">
+        <v>586</v>
+      </c>
+      <c r="E10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" t="s">
+        <v>595</v>
+      </c>
+      <c r="G10" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B11" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="C11" t="s">
+        <v>561</v>
+      </c>
+      <c r="D11" t="s">
+        <v>588</v>
+      </c>
+      <c r="E11" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" t="s">
+        <v>596</v>
+      </c>
+      <c r="G11" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B12" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="C12" t="s">
+        <v>562</v>
+      </c>
+      <c r="D12" t="s">
+        <v>588</v>
+      </c>
+      <c r="E12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" t="s">
+        <v>597</v>
+      </c>
+      <c r="G12" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B13" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="C13" t="s">
+        <v>563</v>
+      </c>
+      <c r="D13" t="s">
+        <v>584</v>
+      </c>
+      <c r="E13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" t="s">
+        <v>597</v>
+      </c>
+      <c r="G13" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B14" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="C14" t="s">
+        <v>564</v>
+      </c>
+      <c r="D14" t="s">
+        <v>584</v>
+      </c>
+      <c r="E14" t="s">
+        <v>22</v>
+      </c>
+      <c r="F14" t="s">
+        <v>597</v>
+      </c>
+      <c r="G14" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B15" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="C15" t="s">
+        <v>565</v>
+      </c>
+      <c r="D15" t="s">
+        <v>585</v>
+      </c>
+      <c r="E15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" t="s">
+        <v>597</v>
+      </c>
+      <c r="G15" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B16" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="C16" t="s">
+        <v>566</v>
+      </c>
+      <c r="D16" t="s">
+        <v>586</v>
+      </c>
+      <c r="E16" t="s">
+        <v>22</v>
+      </c>
+      <c r="F16" t="s">
+        <v>597</v>
+      </c>
+      <c r="G16" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B17" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="C17" t="s">
+        <v>567</v>
+      </c>
+      <c r="D17" t="s">
+        <v>586</v>
+      </c>
+      <c r="E17" t="s">
+        <v>22</v>
+      </c>
+      <c r="F17" t="s">
+        <v>597</v>
+      </c>
+      <c r="G17" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B18" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="C18" t="s">
+        <v>568</v>
+      </c>
+      <c r="D18" t="s">
+        <v>586</v>
+      </c>
+      <c r="E18" t="s">
+        <v>22</v>
+      </c>
+      <c r="F18" t="s">
+        <v>597</v>
+      </c>
+      <c r="G18" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B19" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="C19" t="s">
+        <v>564</v>
+      </c>
+      <c r="D19" t="s">
+        <v>586</v>
+      </c>
+      <c r="E19" t="s">
+        <v>22</v>
+      </c>
+      <c r="F19" t="s">
+        <v>597</v>
+      </c>
+      <c r="G19" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B20" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="C20" t="s">
+        <v>564</v>
+      </c>
+      <c r="D20" t="s">
+        <v>588</v>
+      </c>
+      <c r="E20" t="s">
+        <v>22</v>
+      </c>
+      <c r="F20" t="s">
+        <v>597</v>
+      </c>
+      <c r="G20" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B21" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="C21" t="s">
+        <v>569</v>
+      </c>
+      <c r="D21" t="s">
+        <v>588</v>
+      </c>
+      <c r="E21" t="s">
+        <v>22</v>
+      </c>
+      <c r="F21" t="s">
+        <v>597</v>
+      </c>
+      <c r="G21" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B22" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="C22" t="s">
+        <v>564</v>
+      </c>
+      <c r="D22" t="s">
+        <v>584</v>
+      </c>
+      <c r="E22" t="s">
+        <v>22</v>
+      </c>
+      <c r="F22" t="s">
+        <v>597</v>
+      </c>
+      <c r="G22" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B23" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="C23" t="s">
+        <v>570</v>
+      </c>
+      <c r="D23" t="s">
+        <v>585</v>
+      </c>
+      <c r="E23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B24" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="C24" t="s">
+        <v>571</v>
+      </c>
+      <c r="D24" t="s">
+        <v>585</v>
+      </c>
+      <c r="E24" t="s">
+        <v>22</v>
+      </c>
+      <c r="F24" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B25" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="C25" t="s">
+        <v>572</v>
+      </c>
+      <c r="D25">
+        <v>2024</v>
+      </c>
+      <c r="E25" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B26" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="C26" t="s">
+        <v>573</v>
+      </c>
+      <c r="D26">
+        <v>2025</v>
+      </c>
+      <c r="E26" t="s">
+        <v>22</v>
+      </c>
+      <c r="F26" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B27" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="C27" t="s">
+        <v>574</v>
+      </c>
+      <c r="D27">
+        <v>2025</v>
+      </c>
+      <c r="E27" t="s">
+        <v>22</v>
+      </c>
+      <c r="F27" t="s">
+        <v>600</v>
+      </c>
+      <c r="G27" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B28" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="C28" t="s">
+        <v>575</v>
+      </c>
+      <c r="D28">
+        <v>2024</v>
+      </c>
+      <c r="E28" t="s">
+        <v>22</v>
+      </c>
+      <c r="F28" t="s">
+        <v>601</v>
+      </c>
+      <c r="G28" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B29" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="C29" t="s">
+        <v>576</v>
+      </c>
+      <c r="D29">
+        <v>2023</v>
+      </c>
+      <c r="E29" t="s">
+        <v>22</v>
+      </c>
+      <c r="F29" t="s">
+        <v>601</v>
+      </c>
+      <c r="G29" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B30" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="C30" t="s">
+        <v>577</v>
+      </c>
+      <c r="D30">
+        <v>2026</v>
+      </c>
+      <c r="E30" t="s">
+        <v>22</v>
+      </c>
+      <c r="F30" t="s">
+        <v>602</v>
+      </c>
+      <c r="G30" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B31" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="C31" t="s">
+        <v>578</v>
+      </c>
+      <c r="D31">
+        <v>2026</v>
+      </c>
+      <c r="E31" t="s">
+        <v>22</v>
+      </c>
+      <c r="F31" t="s">
+        <v>602</v>
+      </c>
+      <c r="G31" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B32" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="C32" t="s">
+        <v>579</v>
+      </c>
+      <c r="D32">
+        <v>2025</v>
+      </c>
+      <c r="E32" t="s">
+        <v>22</v>
+      </c>
+      <c r="F32" t="s">
+        <v>600</v>
+      </c>
+      <c r="G32" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B33" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="C33" t="s">
+        <v>580</v>
+      </c>
+      <c r="D33">
+        <v>2024</v>
+      </c>
+      <c r="E33" t="s">
+        <v>22</v>
+      </c>
+      <c r="F33" t="s">
+        <v>603</v>
+      </c>
+      <c r="G33" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B34" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="C34" t="s">
+        <v>581</v>
+      </c>
+      <c r="D34">
+        <v>2024</v>
+      </c>
+      <c r="E34" t="s">
+        <v>22</v>
+      </c>
+      <c r="F34" t="s">
+        <v>600</v>
+      </c>
+      <c r="G34" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" ht="145" x14ac:dyDescent="0.35">
+      <c r="B35" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="C35" t="s">
+        <v>582</v>
+      </c>
+      <c r="D35">
+        <v>2024</v>
+      </c>
+      <c r="E35" t="s">
+        <v>22</v>
+      </c>
+      <c r="F35" t="s">
+        <v>604</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B36" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="C36" t="s">
+        <v>583</v>
+      </c>
+      <c r="D36">
+        <v>2023</v>
+      </c>
+      <c r="E36" t="s">
+        <v>22</v>
+      </c>
+      <c r="F36" t="s">
+        <v>590</v>
+      </c>
+      <c r="G36" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B37" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="C37" t="s">
+        <v>639</v>
+      </c>
+      <c r="D37" t="s">
+        <v>584</v>
+      </c>
+      <c r="E37" t="s">
+        <v>40</v>
+      </c>
+      <c r="F37" t="s">
+        <v>655</v>
+      </c>
+      <c r="G37" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B38" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="C38" t="s">
+        <v>640</v>
+      </c>
+      <c r="D38" t="s">
+        <v>586</v>
+      </c>
+      <c r="E38" t="s">
+        <v>40</v>
+      </c>
+      <c r="F38" t="s">
+        <v>656</v>
+      </c>
+      <c r="G38" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B39" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="C39" t="s">
+        <v>641</v>
+      </c>
+      <c r="D39" t="s">
+        <v>588</v>
+      </c>
+      <c r="E39" t="s">
+        <v>40</v>
+      </c>
+      <c r="F39" t="s">
+        <v>655</v>
+      </c>
+      <c r="G39" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="40" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B40" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="C40" t="s">
+        <v>642</v>
+      </c>
+      <c r="D40" t="s">
+        <v>584</v>
+      </c>
+      <c r="E40" t="s">
+        <v>40</v>
+      </c>
+      <c r="F40" t="s">
+        <v>590</v>
+      </c>
+      <c r="G40" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="41" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B41" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="C41" t="s">
+        <v>643</v>
+      </c>
+      <c r="D41" t="s">
+        <v>586</v>
+      </c>
+      <c r="E41" t="s">
+        <v>40</v>
+      </c>
+      <c r="F41" t="s">
+        <v>655</v>
+      </c>
+      <c r="G41" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="42" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B42" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="C42" t="s">
+        <v>644</v>
+      </c>
+      <c r="D42" t="s">
+        <v>586</v>
+      </c>
+      <c r="E42" t="s">
+        <v>40</v>
+      </c>
+      <c r="F42" t="s">
+        <v>657</v>
+      </c>
+      <c r="G42" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="43" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B43" s="2" t="s">
+        <v>627</v>
+      </c>
+      <c r="C43" t="s">
+        <v>645</v>
+      </c>
+      <c r="D43" t="s">
+        <v>586</v>
+      </c>
+      <c r="E43" t="s">
+        <v>40</v>
+      </c>
+      <c r="F43" t="s">
+        <v>657</v>
+      </c>
+      <c r="G43" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="44" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B44" s="2" t="s">
+        <v>628</v>
+      </c>
+      <c r="C44" t="s">
+        <v>644</v>
+      </c>
+      <c r="D44" t="s">
+        <v>588</v>
+      </c>
+      <c r="E44" t="s">
+        <v>40</v>
+      </c>
+      <c r="F44" t="s">
+        <v>658</v>
+      </c>
+      <c r="G44" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="45" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B45" s="2" t="s">
+        <v>629</v>
+      </c>
+      <c r="C45" t="s">
+        <v>646</v>
+      </c>
+      <c r="D45" t="s">
+        <v>584</v>
+      </c>
+      <c r="E45" t="s">
+        <v>40</v>
+      </c>
+      <c r="F45" t="s">
+        <v>659</v>
+      </c>
+      <c r="G45" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="46" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B46" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="C46" t="s">
+        <v>647</v>
+      </c>
+      <c r="D46" t="s">
+        <v>585</v>
+      </c>
+      <c r="E46" t="s">
+        <v>40</v>
+      </c>
+      <c r="F46" t="s">
+        <v>660</v>
+      </c>
+      <c r="G46" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="47" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B47" s="2" t="s">
+        <v>631</v>
+      </c>
+      <c r="C47" t="s">
+        <v>648</v>
+      </c>
+      <c r="D47" t="s">
+        <v>586</v>
+      </c>
+      <c r="E47" t="s">
+        <v>40</v>
+      </c>
+      <c r="F47" t="s">
+        <v>661</v>
+      </c>
+      <c r="G47" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="48" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B48" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="C48" t="s">
+        <v>649</v>
+      </c>
+      <c r="D48" t="s">
+        <v>584</v>
+      </c>
+      <c r="E48" t="s">
+        <v>40</v>
+      </c>
+      <c r="F48" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="49" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B49" s="2" t="s">
+        <v>633</v>
+      </c>
+      <c r="C49" t="s">
+        <v>650</v>
+      </c>
+      <c r="D49" t="s">
+        <v>585</v>
+      </c>
+      <c r="E49" t="s">
+        <v>40</v>
+      </c>
+      <c r="F49" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="50" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B50" s="2" t="s">
+        <v>634</v>
+      </c>
+      <c r="C50" t="s">
+        <v>651</v>
+      </c>
+      <c r="D50" t="s">
+        <v>585</v>
+      </c>
+      <c r="E50" t="s">
+        <v>40</v>
+      </c>
+      <c r="F50" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="51" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B51" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C51" t="s">
+        <v>652</v>
+      </c>
+      <c r="D51" t="s">
+        <v>586</v>
+      </c>
+      <c r="E51" t="s">
+        <v>40</v>
+      </c>
+      <c r="F51" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B52" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="C52" t="s">
+        <v>652</v>
+      </c>
+      <c r="D52" t="s">
+        <v>586</v>
+      </c>
+      <c r="E52" t="s">
+        <v>40</v>
+      </c>
+      <c r="F52" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B53" s="2" t="s">
+        <v>637</v>
+      </c>
+      <c r="C53" t="s">
+        <v>653</v>
+      </c>
+      <c r="D53" t="s">
+        <v>586</v>
+      </c>
+      <c r="E53" t="s">
+        <v>40</v>
+      </c>
+      <c r="F53" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B54" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="C54" t="s">
+        <v>654</v>
+      </c>
+      <c r="D54" t="s">
+        <v>586</v>
+      </c>
+      <c r="E54" t="s">
+        <v>40</v>
+      </c>
+      <c r="F54" t="s">
+        <v>664</v>
       </c>
     </row>
   </sheetData>
@@ -4783,7 +6109,7 @@
         <v>9</v>
       </c>
       <c r="D1" t="s">
-        <v>342</v>
+        <v>305</v>
       </c>
       <c r="E1" t="s">
         <v>8</v>
@@ -4795,7 +6121,7 @@
         <v>13</v>
       </c>
       <c r="H1" t="s">
-        <v>343</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
@@ -4803,22 +6129,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>344</v>
+        <v>307</v>
       </c>
       <c r="C2" t="s">
-        <v>345</v>
+        <v>308</v>
       </c>
       <c r="D2" t="s">
-        <v>346</v>
+        <v>309</v>
       </c>
       <c r="E2" t="s">
-        <v>347</v>
+        <v>310</v>
       </c>
       <c r="G2" t="s">
-        <v>348</v>
+        <v>311</v>
       </c>
       <c r="H2" t="s">
-        <v>349</v>
+        <v>312</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -4826,19 +6152,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>350</v>
+        <v>313</v>
       </c>
       <c r="C3" t="s">
-        <v>351</v>
+        <v>314</v>
       </c>
       <c r="D3" t="s">
-        <v>352</v>
+        <v>315</v>
       </c>
       <c r="E3" t="s">
         <v>34</v>
       </c>
       <c r="H3" t="s">
-        <v>353</v>
+        <v>316</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -4846,19 +6172,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>354</v>
+        <v>317</v>
       </c>
       <c r="C4" t="s">
-        <v>355</v>
+        <v>318</v>
       </c>
       <c r="D4" t="s">
-        <v>356</v>
+        <v>319</v>
       </c>
       <c r="E4" t="s">
-        <v>357</v>
+        <v>320</v>
       </c>
       <c r="G4" t="s">
-        <v>358</v>
+        <v>321</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -4866,16 +6192,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>359</v>
+        <v>322</v>
       </c>
       <c r="C5" t="s">
-        <v>360</v>
+        <v>323</v>
       </c>
       <c r="D5" t="s">
-        <v>361</v>
+        <v>324</v>
       </c>
       <c r="E5" t="s">
-        <v>362</v>
+        <v>325</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -4883,19 +6209,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>363</v>
+        <v>326</v>
       </c>
       <c r="C6" t="s">
-        <v>364</v>
+        <v>327</v>
       </c>
       <c r="D6" t="s">
-        <v>365</v>
+        <v>328</v>
       </c>
       <c r="E6" t="s">
         <v>34</v>
       </c>
       <c r="H6" t="s">
-        <v>366</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -4916,22 +6242,22 @@
         <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>317</v>
+        <v>297</v>
       </c>
       <c r="D1" t="s">
         <v>51</v>
       </c>
       <c r="E1" t="s">
-        <v>282</v>
+        <v>262</v>
       </c>
       <c r="F1" t="s">
-        <v>318</v>
+        <v>298</v>
       </c>
       <c r="G1" t="s">
-        <v>319</v>
+        <v>299</v>
       </c>
       <c r="H1" t="s">
-        <v>320</v>
+        <v>300</v>
       </c>
       <c r="I1" t="s">
         <v>12</v>
@@ -4945,31 +6271,31 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>367</v>
+        <v>330</v>
       </c>
       <c r="C2" t="s">
         <v>71</v>
       </c>
       <c r="D2" t="s">
-        <v>323</v>
+        <v>301</v>
       </c>
       <c r="E2" t="s">
-        <v>368</v>
+        <v>331</v>
       </c>
       <c r="F2" t="s">
-        <v>369</v>
+        <v>332</v>
       </c>
       <c r="G2" t="s">
-        <v>331</v>
+        <v>303</v>
       </c>
       <c r="H2" t="s">
-        <v>370</v>
+        <v>333</v>
       </c>
       <c r="I2" t="s">
-        <v>371</v>
+        <v>334</v>
       </c>
       <c r="J2" t="s">
-        <v>372</v>
+        <v>335</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
@@ -4977,25 +6303,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>373</v>
+        <v>336</v>
       </c>
       <c r="C3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D3" t="s">
-        <v>323</v>
+        <v>301</v>
       </c>
       <c r="E3" t="s">
-        <v>368</v>
+        <v>331</v>
       </c>
       <c r="F3" t="s">
-        <v>374</v>
+        <v>337</v>
       </c>
       <c r="G3" t="s">
-        <v>325</v>
+        <v>302</v>
       </c>
       <c r="H3" t="s">
-        <v>375</v>
+        <v>338</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -5003,28 +6329,28 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>376</v>
+        <v>339</v>
       </c>
       <c r="C4" t="s">
         <v>97</v>
       </c>
       <c r="D4" t="s">
-        <v>335</v>
+        <v>304</v>
       </c>
       <c r="E4" t="s">
-        <v>368</v>
+        <v>331</v>
       </c>
       <c r="F4" t="s">
-        <v>377</v>
+        <v>340</v>
       </c>
       <c r="G4" t="s">
-        <v>331</v>
+        <v>303</v>
       </c>
       <c r="H4" t="s">
-        <v>378</v>
+        <v>341</v>
       </c>
       <c r="I4" t="s">
-        <v>379</v>
+        <v>342</v>
       </c>
     </row>
   </sheetData>

</xml_diff>